<commit_message>
Add comprehensive validation checklist for system modules and integrations
Generate an Excel file containing multiple sheets detailing modules, screens, API endpoints, database tables and columns, integrations, and a validation checklist.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: e70c97c4-e099-455a-b9ae-aa9a0dedb718
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: c74567b4-9049-4a71-84da-65792180c435
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/713657ac-53c6-43a9-97a8-ef2697ef92d9/e70c97c4-e099-455a-b9ae-aa9a0dedb718/M9k368Z
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/gold_erp_validation.xlsx
+++ b/gold_erp_validation.xlsx
@@ -17,18 +17,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
       <scheme val="minor"/>
       <sz val="11"/>
       <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FF1A237E"/>
-      <sz val="9"/>
     </font>
     <font>
       <b/>
@@ -44,9 +39,6 @@
       <color rgb="FF1F3864"/>
       <sz val="9"/>
     </font>
-    <font>
-      <sz val="9"/>
-    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -57,7 +49,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF444444"/>
+        <fgColor rgb="FF1F6B35"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1B4F72"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF7B241C"/>
       </patternFill>
     </fill>
     <fill>
@@ -75,16 +77,6 @@
         <fgColor rgb="FF6D4C41"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF1F6B35"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF1B4F72"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -98,30 +90,28 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -461,7 +451,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B1:B42"/>
+  <dimension ref="A1:A42"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -469,73 +459,53 @@
     <col min="3" max="3" width="34" customWidth="1"/>
     <col min="4" max="4" width="32" customWidth="1"/>
     <col min="5" max="5" width="40" customWidth="1"/>
-    <col min="6" max="6" width="18" customWidth="1"/>
+    <col min="6" max="6" width="16" customWidth="1"/>
     <col min="7" max="7" width="20" customWidth="1"/>
     <col min="8" max="8" width="30" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="2" ht="18" customHeight="1" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B2" s="1"/>
-    </row>
-    <row r="3" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="4" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="6" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="7" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="8" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="9" ht="18" customHeight="1" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B9" s="1"/>
-    </row>
-    <row r="10" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="11" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="12" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="13" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="14" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="15" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="16" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="17" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="18" ht="18" customHeight="1" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B18" s="1"/>
-    </row>
-    <row r="19" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="20" ht="18" customHeight="1" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B20" s="1"/>
-    </row>
-    <row r="21" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="22" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="23" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="24" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="25" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="26" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="27" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="28" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="29" ht="18" customHeight="1" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B29" s="1"/>
-    </row>
-    <row r="30" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="31" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="32" ht="18" customHeight="1" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B32" s="1"/>
-    </row>
-    <row r="33" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="34" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="35" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="36" ht="18" customHeight="1" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B36" s="1"/>
-    </row>
-    <row r="37" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="38" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="39" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="40" ht="18" customHeight="1" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B40" s="1"/>
-    </row>
-    <row r="41" ht="18" customHeight="1" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B41" s="1"/>
-    </row>
-    <row r="42" ht="18" customHeight="1" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B42" s="1"/>
-    </row>
+    <row r="2" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="3" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="4" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="5" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="6" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="7" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="8" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="9" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="10" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="11" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="12" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="13" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="14" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="15" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="16" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="17" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="18" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="19" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="20" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="21" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="22" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="23" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="24" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="25" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="26" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="27" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="28" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="29" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="30" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="31" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="32" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="33" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="34" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="35" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="36" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="37" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="38" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="39" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="40" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="41" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="42" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -549,566 +519,566 @@
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
-    <col min="2" max="2" width="22" customWidth="1"/>
+    <col min="2" max="2" width="20" customWidth="1"/>
     <col min="3" max="3" width="10" customWidth="1"/>
     <col min="4" max="4" width="50" customWidth="1"/>
     <col min="5" max="5" width="45" customWidth="1"/>
-    <col min="6" max="6" width="15" customWidth="1"/>
+    <col min="6" max="6" width="8" customWidth="1"/>
     <col min="7" max="7" width="20" customWidth="1"/>
     <col min="8" max="8" width="30" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="2" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C2" s="2"/>
-    </row>
-    <row r="3" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C3" s="2"/>
-    </row>
-    <row r="4" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C4" s="2"/>
-    </row>
-    <row r="5" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="2" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C2" s="1"/>
+    </row>
+    <row r="3" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C3" s="1"/>
+    </row>
+    <row r="4" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C4" s="1"/>
+    </row>
+    <row r="5" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C5" s="2"/>
     </row>
-    <row r="6" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C6" s="2"/>
-    </row>
-    <row r="7" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C7" s="2"/>
-    </row>
-    <row r="8" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="6" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C6" s="3"/>
+    </row>
+    <row r="7" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C7" s="1"/>
+    </row>
+    <row r="8" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C8" s="2"/>
     </row>
-    <row r="9" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C9" s="2"/>
-    </row>
-    <row r="10" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C10" s="2"/>
-    </row>
-    <row r="11" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C11" s="2"/>
-    </row>
-    <row r="12" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="9" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C9" s="4"/>
+    </row>
+    <row r="10" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C10" s="3"/>
+    </row>
+    <row r="11" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C11" s="1"/>
+    </row>
+    <row r="12" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C12" s="2"/>
     </row>
-    <row r="13" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C13" s="2"/>
-    </row>
-    <row r="14" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C14" s="2"/>
-    </row>
-    <row r="15" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C15" s="2"/>
-    </row>
-    <row r="16" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="13" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C13" s="4"/>
+    </row>
+    <row r="14" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C14" s="3"/>
+    </row>
+    <row r="15" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C15" s="1"/>
+    </row>
+    <row r="16" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C16" s="2"/>
     </row>
-    <row r="17" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C17" s="2"/>
-    </row>
-    <row r="18" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C18" s="2"/>
-    </row>
-    <row r="19" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C19" s="2"/>
-    </row>
-    <row r="20" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="17" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C17" s="4"/>
+    </row>
+    <row r="18" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C18" s="1"/>
+    </row>
+    <row r="19" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C19" s="1"/>
+    </row>
+    <row r="20" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C20" s="2"/>
     </row>
-    <row r="21" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C21" s="2"/>
-    </row>
-    <row r="22" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C22" s="2"/>
-    </row>
-    <row r="23" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C23" s="2"/>
-    </row>
-    <row r="24" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C24" s="2"/>
-    </row>
-    <row r="25" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C25" s="2"/>
-    </row>
-    <row r="26" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C26" s="2"/>
-    </row>
-    <row r="27" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C27" s="2"/>
-    </row>
-    <row r="28" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C28" s="2"/>
-    </row>
-    <row r="29" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C29" s="2"/>
-    </row>
-    <row r="30" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C30" s="2"/>
-    </row>
-    <row r="31" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C31" s="2"/>
-    </row>
-    <row r="32" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C32" s="2"/>
-    </row>
-    <row r="33" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="21" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C21" s="1"/>
+    </row>
+    <row r="22" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C22" s="1"/>
+    </row>
+    <row r="23" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C23" s="1"/>
+    </row>
+    <row r="24" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C24" s="1"/>
+    </row>
+    <row r="25" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C25" s="1"/>
+    </row>
+    <row r="26" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C26" s="1"/>
+    </row>
+    <row r="27" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C27" s="1"/>
+    </row>
+    <row r="28" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C28" s="1"/>
+    </row>
+    <row r="29" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C29" s="1"/>
+    </row>
+    <row r="30" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C30" s="1"/>
+    </row>
+    <row r="31" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C31" s="1"/>
+    </row>
+    <row r="32" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C32" s="1"/>
+    </row>
+    <row r="33" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C33" s="2"/>
     </row>
-    <row r="34" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C34" s="2"/>
-    </row>
-    <row r="35" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C35" s="2"/>
-    </row>
-    <row r="36" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C36" s="2"/>
-    </row>
-    <row r="37" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="34" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C34" s="4"/>
+    </row>
+    <row r="35" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C35" s="3"/>
+    </row>
+    <row r="36" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C36" s="1"/>
+    </row>
+    <row r="37" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C37" s="2"/>
     </row>
-    <row r="38" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C38" s="2"/>
-    </row>
-    <row r="39" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C39" s="2"/>
-    </row>
-    <row r="40" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C40" s="2"/>
-    </row>
-    <row r="41" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C41" s="2"/>
-    </row>
-    <row r="42" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="38" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C38" s="1"/>
+    </row>
+    <row r="39" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C39" s="4"/>
+    </row>
+    <row r="40" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C40" s="4"/>
+    </row>
+    <row r="41" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C41" s="1"/>
+    </row>
+    <row r="42" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C42" s="2"/>
     </row>
-    <row r="43" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C43" s="2"/>
-    </row>
-    <row r="44" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C44" s="2"/>
-    </row>
-    <row r="45" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="43" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C43" s="4"/>
+    </row>
+    <row r="44" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C44" s="1"/>
+    </row>
+    <row r="45" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C45" s="2"/>
     </row>
-    <row r="46" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C46" s="2"/>
-    </row>
-    <row r="47" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C47" s="2"/>
-    </row>
-    <row r="48" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="46" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C46" s="4"/>
+    </row>
+    <row r="47" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C47" s="1"/>
+    </row>
+    <row r="48" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C48" s="2"/>
     </row>
-    <row r="49" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C49" s="2"/>
-    </row>
-    <row r="50" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C50" s="2"/>
-    </row>
-    <row r="51" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="49" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C49" s="4"/>
+    </row>
+    <row r="50" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C50" s="1"/>
+    </row>
+    <row r="51" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C51" s="2"/>
     </row>
-    <row r="52" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C52" s="2"/>
-    </row>
-    <row r="53" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C53" s="2"/>
-    </row>
-    <row r="54" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="52" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C52" s="4"/>
+    </row>
+    <row r="53" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C53" s="1"/>
+    </row>
+    <row r="54" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C54" s="2"/>
     </row>
-    <row r="55" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C55" s="2"/>
-    </row>
-    <row r="56" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="55" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C55" s="1"/>
+    </row>
+    <row r="56" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C56" s="2"/>
     </row>
-    <row r="57" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C57" s="2"/>
-    </row>
-    <row r="58" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="57" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C57" s="1"/>
+    </row>
+    <row r="58" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C58" s="2"/>
     </row>
-    <row r="59" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C59" s="2"/>
-    </row>
-    <row r="60" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C60" s="2"/>
-    </row>
-    <row r="61" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="59" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C59" s="4"/>
+    </row>
+    <row r="60" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C60" s="1"/>
+    </row>
+    <row r="61" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C61" s="2"/>
     </row>
-    <row r="62" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C62" s="2"/>
-    </row>
-    <row r="63" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="62" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C62" s="1"/>
+    </row>
+    <row r="63" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C63" s="2"/>
     </row>
-    <row r="64" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C64" s="2"/>
-    </row>
-    <row r="65" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="64" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C64" s="1"/>
+    </row>
+    <row r="65" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C65" s="2"/>
     </row>
-    <row r="66" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C66" s="2"/>
-    </row>
-    <row r="67" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="66" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C66" s="1"/>
+    </row>
+    <row r="67" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C67" s="2"/>
     </row>
-    <row r="68" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C68" s="2"/>
-    </row>
-    <row r="69" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="68" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C68" s="1"/>
+    </row>
+    <row r="69" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C69" s="2"/>
     </row>
-    <row r="70" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C70" s="2"/>
-    </row>
-    <row r="71" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C71" s="2"/>
-    </row>
-    <row r="72" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C72" s="2"/>
-    </row>
-    <row r="73" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="70" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C70" s="4"/>
+    </row>
+    <row r="71" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C71" s="3"/>
+    </row>
+    <row r="72" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C72" s="1"/>
+    </row>
+    <row r="73" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C73" s="2"/>
     </row>
-    <row r="74" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C74" s="2"/>
-    </row>
-    <row r="75" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C75" s="2"/>
-    </row>
-    <row r="76" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="74" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C74" s="4"/>
+    </row>
+    <row r="75" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C75" s="1"/>
+    </row>
+    <row r="76" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C76" s="2"/>
     </row>
-    <row r="77" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C77" s="2"/>
-    </row>
-    <row r="78" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C78" s="2"/>
-    </row>
-    <row r="79" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="77" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C77" s="4"/>
+    </row>
+    <row r="78" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C78" s="1"/>
+    </row>
+    <row r="79" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C79" s="2"/>
     </row>
-    <row r="80" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C80" s="2"/>
-    </row>
-    <row r="81" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C81" s="2"/>
-    </row>
-    <row r="82" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="80" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C80" s="4"/>
+    </row>
+    <row r="81" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C81" s="1"/>
+    </row>
+    <row r="82" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C82" s="2"/>
     </row>
-    <row r="83" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C83" s="2"/>
-    </row>
-    <row r="84" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C84" s="2"/>
-    </row>
-    <row r="85" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="83" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C83" s="4"/>
+    </row>
+    <row r="84" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C84" s="1"/>
+    </row>
+    <row r="85" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C85" s="2"/>
     </row>
-    <row r="86" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C86" s="2"/>
-    </row>
-    <row r="87" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C87" s="2"/>
-    </row>
-    <row r="88" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="86" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C86" s="4"/>
+    </row>
+    <row r="87" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C87" s="1"/>
+    </row>
+    <row r="88" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C88" s="2"/>
     </row>
-    <row r="89" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C89" s="2"/>
-    </row>
-    <row r="90" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C90" s="2"/>
-    </row>
-    <row r="91" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="89" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C89" s="4"/>
+    </row>
+    <row r="90" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C90" s="1"/>
+    </row>
+    <row r="91" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C91" s="2"/>
     </row>
-    <row r="92" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C92" s="2"/>
-    </row>
-    <row r="93" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="92" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C92" s="1"/>
+    </row>
+    <row r="93" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C93" s="2"/>
     </row>
-    <row r="94" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="94" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C94" s="2"/>
     </row>
-    <row r="95" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C95" s="2"/>
-    </row>
-    <row r="96" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="95" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C95" s="1"/>
+    </row>
+    <row r="96" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C96" s="2"/>
     </row>
-    <row r="97" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C97" s="2"/>
-    </row>
-    <row r="98" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C98" s="2"/>
-    </row>
-    <row r="99" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="97" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C97" s="4"/>
+    </row>
+    <row r="98" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C98" s="1"/>
+    </row>
+    <row r="99" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C99" s="2"/>
     </row>
-    <row r="100" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C100" s="2"/>
-    </row>
-    <row r="101" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C101" s="2"/>
-    </row>
-    <row r="102" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="100" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C100" s="4"/>
+    </row>
+    <row r="101" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C101" s="1"/>
+    </row>
+    <row r="102" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C102" s="2"/>
     </row>
-    <row r="103" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C103" s="2"/>
-    </row>
-    <row r="104" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="103" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C103" s="1"/>
+    </row>
+    <row r="104" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C104" s="2"/>
     </row>
-    <row r="105" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C105" s="2"/>
-    </row>
-    <row r="106" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C106" s="2"/>
-    </row>
-    <row r="107" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C107" s="2"/>
-    </row>
-    <row r="108" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="105" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C105" s="4"/>
+    </row>
+    <row r="106" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C106" s="1"/>
+    </row>
+    <row r="107" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C107" s="1"/>
+    </row>
+    <row r="108" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C108" s="2"/>
     </row>
-    <row r="109" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C109" s="2"/>
-    </row>
-    <row r="110" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C110" s="2"/>
-    </row>
-    <row r="111" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="109" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C109" s="3"/>
+    </row>
+    <row r="110" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C110" s="1"/>
+    </row>
+    <row r="111" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C111" s="2"/>
     </row>
-    <row r="112" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C112" s="2"/>
-    </row>
-    <row r="113" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C113" s="2"/>
-    </row>
-    <row r="114" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="112" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C112" s="4"/>
+    </row>
+    <row r="113" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C113" s="1"/>
+    </row>
+    <row r="114" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C114" s="2"/>
     </row>
-    <row r="115" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C115" s="2"/>
-    </row>
-    <row r="116" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C116" s="2"/>
-    </row>
-    <row r="117" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="115" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C115" s="4"/>
+    </row>
+    <row r="116" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C116" s="1"/>
+    </row>
+    <row r="117" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C117" s="2"/>
     </row>
-    <row r="118" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C118" s="2"/>
-    </row>
-    <row r="119" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C119" s="2"/>
-    </row>
-    <row r="120" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="118" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C118" s="4"/>
+    </row>
+    <row r="119" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C119" s="1"/>
+    </row>
+    <row r="120" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C120" s="2"/>
     </row>
-    <row r="121" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="121" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C121" s="2"/>
     </row>
-    <row r="122" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C122" s="2"/>
-    </row>
-    <row r="123" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C123" s="2"/>
-    </row>
-    <row r="124" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C124" s="2"/>
-    </row>
-    <row r="125" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="122" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C122" s="1"/>
+    </row>
+    <row r="123" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C123" s="1"/>
+    </row>
+    <row r="124" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C124" s="1"/>
+    </row>
+    <row r="125" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C125" s="2"/>
     </row>
-    <row r="126" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C126" s="2"/>
-    </row>
-    <row r="127" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="126" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C126" s="1"/>
+    </row>
+    <row r="127" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C127" s="2"/>
     </row>
-    <row r="128" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C128" s="2"/>
-    </row>
-    <row r="129" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="128" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C128" s="1"/>
+    </row>
+    <row r="129" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C129" s="2"/>
     </row>
-    <row r="130" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C130" s="2"/>
-    </row>
-    <row r="131" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="130" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C130" s="4"/>
+    </row>
+    <row r="131" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C131" s="2"/>
     </row>
-    <row r="132" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C132" s="2"/>
-    </row>
-    <row r="133" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C133" s="2"/>
-    </row>
-    <row r="134" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C134" s="2"/>
-    </row>
-    <row r="135" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C135" s="2"/>
-    </row>
-    <row r="136" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C136" s="2"/>
-    </row>
-    <row r="137" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="132" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C132" s="1"/>
+    </row>
+    <row r="133" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C133" s="1"/>
+    </row>
+    <row r="134" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C134" s="1"/>
+    </row>
+    <row r="135" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C135" s="1"/>
+    </row>
+    <row r="136" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C136" s="1"/>
+    </row>
+    <row r="137" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C137" s="2"/>
     </row>
-    <row r="138" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C138" s="2"/>
-    </row>
-    <row r="139" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C139" s="2"/>
-    </row>
-    <row r="140" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C140" s="2"/>
-    </row>
-    <row r="141" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C141" s="2"/>
-    </row>
-    <row r="142" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C142" s="2"/>
-    </row>
-    <row r="143" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C143" s="2"/>
-    </row>
-    <row r="144" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C144" s="2"/>
-    </row>
-    <row r="145" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="138" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C138" s="4"/>
+    </row>
+    <row r="139" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C139" s="1"/>
+    </row>
+    <row r="140" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C140" s="1"/>
+    </row>
+    <row r="141" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C141" s="4"/>
+    </row>
+    <row r="142" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C142" s="1"/>
+    </row>
+    <row r="143" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C143" s="4"/>
+    </row>
+    <row r="144" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C144" s="1"/>
+    </row>
+    <row r="145" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C145" s="2"/>
     </row>
-    <row r="146" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C146" s="2"/>
-    </row>
-    <row r="147" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C147" s="2"/>
-    </row>
-    <row r="148" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="146" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C146" s="1"/>
+    </row>
+    <row r="147" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C147" s="4"/>
+    </row>
+    <row r="148" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C148" s="2"/>
     </row>
-    <row r="149" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C149" s="2"/>
-    </row>
-    <row r="150" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="149" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C149" s="1"/>
+    </row>
+    <row r="150" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C150" s="2"/>
     </row>
-    <row r="151" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C151" s="2"/>
-    </row>
-    <row r="152" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="151" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C151" s="1"/>
+    </row>
+    <row r="152" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C152" s="2"/>
     </row>
-    <row r="153" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C153" s="2"/>
-    </row>
-    <row r="154" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="153" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C153" s="1"/>
+    </row>
+    <row r="154" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C154" s="2"/>
     </row>
-    <row r="155" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C155" s="2"/>
-    </row>
-    <row r="156" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C156" s="2"/>
-    </row>
-    <row r="157" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="155" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C155" s="4"/>
+    </row>
+    <row r="156" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C156" s="1"/>
+    </row>
+    <row r="157" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C157" s="2"/>
     </row>
-    <row r="158" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C158" s="2"/>
-    </row>
-    <row r="159" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C159" s="2"/>
-    </row>
-    <row r="160" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="158" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C158" s="4"/>
+    </row>
+    <row r="159" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C159" s="1"/>
+    </row>
+    <row r="160" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C160" s="2"/>
     </row>
-    <row r="161" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C161" s="2"/>
-    </row>
-    <row r="162" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C162" s="2"/>
-    </row>
-    <row r="163" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C163" s="2"/>
-    </row>
-    <row r="164" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="161" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C161" s="4"/>
+    </row>
+    <row r="162" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C162" s="1"/>
+    </row>
+    <row r="163" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C163" s="1"/>
+    </row>
+    <row r="164" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C164" s="2"/>
     </row>
-    <row r="165" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C165" s="2"/>
-    </row>
-    <row r="166" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="165" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C165" s="1"/>
+    </row>
+    <row r="166" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C166" s="2"/>
     </row>
-    <row r="167" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C167" s="2"/>
-    </row>
-    <row r="168" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C168" s="2"/>
-    </row>
-    <row r="169" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="167" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C167" s="1"/>
+    </row>
+    <row r="168" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C168" s="1"/>
+    </row>
+    <row r="169" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C169" s="2"/>
     </row>
-    <row r="170" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C170" s="2"/>
-    </row>
-    <row r="171" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="170" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C170" s="1"/>
+    </row>
+    <row r="171" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C171" s="2"/>
     </row>
-    <row r="172" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C172" s="2"/>
-    </row>
-    <row r="173" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="172" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C172" s="1"/>
+    </row>
+    <row r="173" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C173" s="2"/>
     </row>
-    <row r="174" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C174" s="2"/>
-    </row>
-    <row r="175" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C175" s="2"/>
-    </row>
-    <row r="176" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C176" s="2"/>
-    </row>
-    <row r="177" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C177" s="2"/>
-    </row>
-    <row r="178" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C178" s="2"/>
-    </row>
-    <row r="179" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C179" s="2"/>
-    </row>
-    <row r="180" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C180" s="2"/>
-    </row>
-    <row r="181" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C181" s="2"/>
-    </row>
-    <row r="182" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C182" s="2"/>
-    </row>
-    <row r="183" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C183" s="2"/>
-    </row>
-    <row r="184" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C184" s="2"/>
-    </row>
-    <row r="185" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="174" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C174" s="1"/>
+    </row>
+    <row r="175" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C175" s="4"/>
+    </row>
+    <row r="176" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C176" s="1"/>
+    </row>
+    <row r="177" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C177" s="4"/>
+    </row>
+    <row r="178" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C178" s="1"/>
+    </row>
+    <row r="179" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C179" s="4"/>
+    </row>
+    <row r="180" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C180" s="1"/>
+    </row>
+    <row r="181" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C181" s="4"/>
+    </row>
+    <row r="182" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C182" s="1"/>
+    </row>
+    <row r="183" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C183" s="4"/>
+    </row>
+    <row r="184" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C184" s="1"/>
+    </row>
+    <row r="185" ht="17" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C185" s="2"/>
     </row>
   </sheetData>
@@ -1120,15 +1090,17 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A605"/>
+  <dimension ref="A1:A594"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
-    <col min="2" max="2" width="24" customWidth="1"/>
-    <col min="3" max="4" width="34" customWidth="1"/>
+    <col min="2" max="2" width="22" customWidth="1"/>
+    <col min="3" max="4" width="32" customWidth="1"/>
     <col min="5" max="5" width="22" customWidth="1"/>
     <col min="6" max="6" width="10" customWidth="1"/>
-    <col min="7" max="7" width="38" customWidth="1"/>
+    <col min="7" max="7" width="40" customWidth="1"/>
+    <col min="8" max="8" width="20" customWidth="1"/>
+    <col min="9" max="9" width="25" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -1725,19 +1697,8 @@
     <row r="592" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="593" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="594" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="595" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="596" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="597" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="598" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="599" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="600" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="601" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="602" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="603" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="604" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="605" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <autoFilter ref="A1:G1"/>
+  <autoFilter ref="A1:I1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -1750,9 +1711,9 @@
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
-    <col min="3" max="3" width="22" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
     <col min="4" max="4" width="52" customWidth="1"/>
-    <col min="5" max="5" width="32" customWidth="1"/>
+    <col min="5" max="5" width="30" customWidth="1"/>
     <col min="6" max="6" width="44" customWidth="1"/>
     <col min="7" max="7" width="16" customWidth="1"/>
     <col min="8" max="8" width="20" customWidth="1"/>
@@ -1760,53 +1721,53 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="2" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
-      <c r="G2" s="3"/>
-    </row>
-    <row r="3" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
-      <c r="G3" s="3"/>
-    </row>
-    <row r="4" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
-      <c r="G4" s="3"/>
-    </row>
-    <row r="5" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
-      <c r="G5" s="4"/>
-    </row>
-    <row r="6" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
-      <c r="G6" s="5"/>
-    </row>
-    <row r="7" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
-      <c r="G7" s="6"/>
-    </row>
-    <row r="8" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
-      <c r="G8" s="6"/>
-    </row>
-    <row r="9" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
-      <c r="G9" s="6"/>
-    </row>
-    <row r="10" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
-      <c r="G10" s="3"/>
-    </row>
-    <row r="11" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
-      <c r="G11" s="3"/>
-    </row>
-    <row r="12" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
-      <c r="G12" s="3"/>
-    </row>
-    <row r="13" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
-      <c r="G13" s="3"/>
-    </row>
-    <row r="14" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
-      <c r="G14" s="6"/>
-    </row>
-    <row r="15" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
-      <c r="G15" s="7"/>
-    </row>
-    <row r="16" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
-      <c r="G16" s="6"/>
-    </row>
-    <row r="17" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
-      <c r="G17" s="6"/>
+    <row r="2" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G2" s="4"/>
+    </row>
+    <row r="3" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G3" s="4"/>
+    </row>
+    <row r="4" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G4" s="4"/>
+    </row>
+    <row r="5" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G5" s="5"/>
+    </row>
+    <row r="6" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G6" s="6"/>
+    </row>
+    <row r="7" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G7" s="1"/>
+    </row>
+    <row r="8" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G8" s="1"/>
+    </row>
+    <row r="9" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G9" s="1"/>
+    </row>
+    <row r="10" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G10" s="4"/>
+    </row>
+    <row r="11" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G11" s="4"/>
+    </row>
+    <row r="12" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G12" s="4"/>
+    </row>
+    <row r="13" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G13" s="4"/>
+    </row>
+    <row r="14" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G14" s="1"/>
+    </row>
+    <row r="15" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G15" s="1"/>
+    </row>
+    <row r="16" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G16" s="2"/>
+    </row>
+    <row r="17" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G17" s="1"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
@@ -1822,87 +1783,87 @@
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
-    <col min="3" max="4" width="50" customWidth="1"/>
-    <col min="5" max="5" width="18" customWidth="1"/>
+    <col min="3" max="4" width="52" customWidth="1"/>
+    <col min="5" max="5" width="16" customWidth="1"/>
     <col min="6" max="6" width="14" customWidth="1"/>
     <col min="7" max="7" width="16" customWidth="1"/>
     <col min="8" max="8" width="40" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="2" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="3" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="4" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="5" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="6" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="7" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="8" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="9" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="10" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="11" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="12" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="13" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="14" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="15" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="16" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="17" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="18" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="19" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="20" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="21" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="22" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="23" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="24" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="25" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="26" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="27" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="28" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="29" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="30" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="31" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="32" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="33" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="34" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="35" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="36" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="37" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="38" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="39" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="40" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="41" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="42" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="43" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="44" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="45" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="46" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="47" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="48" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="49" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="50" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="51" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="52" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="53" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="54" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="55" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="56" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="57" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="58" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="59" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="60" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="61" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="62" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="63" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="64" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="65" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="66" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="67" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="68" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="69" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="70" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="71" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="72" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="73" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
-    <row r="74" ht="18" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="2" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="3" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="4" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="5" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="6" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="7" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="8" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="9" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="10" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="11" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="12" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="13" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="14" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="15" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="16" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="17" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="18" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="19" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="20" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="21" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="22" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="23" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="24" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="25" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="26" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="27" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="28" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="29" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="30" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="31" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="32" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="33" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="34" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="35" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="36" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="37" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="38" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="39" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="40" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="41" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="42" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="43" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="44" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="45" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="46" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="47" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="48" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="49" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="50" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="51" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="52" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="53" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="54" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="55" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="56" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="57" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="58" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="59" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="60" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="61" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="62" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="63" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="64" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="65" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="66" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="67" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="68" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="69" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="70" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="71" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="72" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="73" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="74" ht="17" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <dataValidations count="2">
@@ -1920,86 +1881,63 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B25"/>
+  <dimension ref="A1:B26"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="48" customWidth="1"/>
-    <col min="2" max="2" width="30" customWidth="1"/>
+    <col min="1" max="1" width="50" customWidth="1"/>
+    <col min="2" max="2" width="35" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="2" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="3" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="8"/>
-      <c r="B3" s="9"/>
-    </row>
-    <row r="4" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="8"/>
-      <c r="B4" s="9"/>
-    </row>
-    <row r="5" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="8"/>
-      <c r="B5" s="9"/>
-    </row>
-    <row r="6" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="8"/>
-      <c r="B6" s="9"/>
-    </row>
-    <row r="7" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="8"/>
-      <c r="B7" s="9"/>
-    </row>
-    <row r="8" ht="18" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A8" s="10"/>
-    </row>
-    <row r="9" ht="18" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A9" s="10"/>
-    </row>
-    <row r="10" ht="18" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A10" s="10"/>
-    </row>
-    <row r="11" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="12" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="8"/>
-      <c r="B12" s="9"/>
-    </row>
-    <row r="13" ht="18" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A13" s="10"/>
-    </row>
-    <row r="14" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="15" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" s="8"/>
-      <c r="B15" s="9"/>
-    </row>
-    <row r="16" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" s="8"/>
-      <c r="B16" s="9"/>
-    </row>
-    <row r="17" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="8"/>
-      <c r="B17" s="9"/>
-    </row>
-    <row r="18" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" s="8"/>
-      <c r="B18" s="9"/>
-    </row>
-    <row r="19" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="20" ht="18" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A20" s="10"/>
-    </row>
-    <row r="21" ht="18" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A21" s="10"/>
-    </row>
-    <row r="22" ht="18" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A22" s="10"/>
-    </row>
-    <row r="23" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="24" ht="18" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A24" s="10"/>
-    </row>
-    <row r="25" ht="18" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A25" s="10"/>
-    </row>
+    <row r="2" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="3" ht="17" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="7"/>
+      <c r="B3" s="8"/>
+    </row>
+    <row r="4" ht="17" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="7"/>
+      <c r="B4" s="8"/>
+    </row>
+    <row r="5" ht="17" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="7"/>
+      <c r="B5" s="8"/>
+    </row>
+    <row r="6" ht="17" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="7"/>
+      <c r="B6" s="8"/>
+    </row>
+    <row r="7" ht="17" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="7"/>
+      <c r="B7" s="8"/>
+    </row>
+    <row r="8" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="9" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="10" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="11" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="12" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="13" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="14" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="15" ht="17" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" s="7"/>
+      <c r="B15" s="8"/>
+    </row>
+    <row r="16" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="17" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="18" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="19" ht="17" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" s="7"/>
+      <c r="B19" s="8"/>
+    </row>
+    <row r="20" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="21" ht="17" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" s="7"/>
+      <c r="B21" s="8"/>
+    </row>
+    <row r="22" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="23" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="24" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="25" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="26" ht="17" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>